<commit_message>
Remove em dashes project-wide; add plain-language PDF project explainer
</commit_message>
<xml_diff>
--- a/data/bi_exports/compliance_audit_workbook.xlsx
+++ b/data/bi_exports/compliance_audit_workbook.xlsx
@@ -76,7 +76,7 @@
     <t xml:space="preserve">OK</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-10 05:54</t>
+    <t xml:space="preserve">2026-07-10 06:01</t>
   </si>
   <si>
     <t xml:space="preserve">LEDGER-002</t>
@@ -85,13 +85,13 @@
     <t xml:space="preserve">LEDGER-003</t>
   </si>
   <si>
-    <t xml:space="preserve">Counterparty Identification (Global — ISO 17442)</t>
+    <t xml:space="preserve">Counterparty Identification (Global - ISO 17442)</t>
   </si>
   <si>
     <t xml:space="preserve">REPORT-001</t>
   </si>
   <si>
-    <t xml:space="preserve">EU — ESMA / EMIR &amp; MiFID II</t>
+    <t xml:space="preserve">EU - ESMA / EMIR &amp; MiFID II</t>
   </si>
   <si>
     <t xml:space="preserve">CDE-001</t>
@@ -100,13 +100,13 @@
     <t xml:space="preserve">TXN-1002</t>
   </si>
   <si>
-    <t xml:space="preserve">US — CFTC / SEC (Dodd-Frank Title VII)</t>
+    <t xml:space="preserve">US - CFTC / SEC (Dodd-Frank Title VII)</t>
   </si>
   <si>
     <t xml:space="preserve">TXN-1003</t>
   </si>
   <si>
-    <t xml:space="preserve">APAC — ASIC / HKMA-SFC / MAS</t>
+    <t xml:space="preserve">APAC - ASIC / HKMA-SFC / MAS</t>
   </si>
   <si>
     <t xml:space="preserve">TXN-1004</t>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported 3 day(s) after the US T+0 deadline (US — CFTC / SEC (Dodd-Frank Title VII)).</t>
+    <t xml:space="preserve">Reported 3 day(s) after the US T+0 deadline (US - CFTC / SEC (Dodd-Frank Title VII)).</t>
   </si>
   <si>
     <t xml:space="preserve">TXN-1006</t>
@@ -199,7 +199,7 @@
     <t xml:space="preserve">TXN-1022</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported 2 day(s) after the EU T+1 deadline (EU — ESMA / EMIR &amp; MiFID II).</t>
+    <t xml:space="preserve">Reported 2 day(s) after the EU T+1 deadline (EU - ESMA / EMIR &amp; MiFID II).</t>
   </si>
   <si>
     <t xml:space="preserve">TXN-1023</t>
@@ -217,7 +217,7 @@
     <t xml:space="preserve">TXN-1027</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported 1 day(s) after the APAC T+2 deadline (APAC — ASIC / HKMA-SFC / MAS).</t>
+    <t xml:space="preserve">Reported 1 day(s) after the APAC T+2 deadline (APAC - ASIC / HKMA-SFC / MAS).</t>
   </si>
   <si>
     <t xml:space="preserve">TXN-1028</t>

</xml_diff>